<commit_message>
added worksheets by name
</commit_message>
<xml_diff>
--- a/Blackjack use case specification.xlsx
+++ b/Blackjack use case specification.xlsx
@@ -8,14 +8,18 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pcooper\Education\Classes\202601 Spring\CS401\Code\CS401_Blackjack\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C16DC788-3386-47C5-9448-C7F098BC8595}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CB506E6-E09E-4E8D-B916-E2C4FB22F7AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{DE0262C4-FE9D-4F25-BADD-B2B186F6EC17}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="6" xr2:uid="{DE0262C4-FE9D-4F25-BADD-B2B186F6EC17}"/>
   </bookViews>
   <sheets>
-    <sheet name="Use case" sheetId="1" r:id="rId1"/>
+    <sheet name="Use case template" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet3" sheetId="3" r:id="rId2"/>
     <sheet name="Permissions" sheetId="2" r:id="rId3"/>
+    <sheet name="Blake" sheetId="4" r:id="rId4"/>
+    <sheet name="Nick" sheetId="5" r:id="rId5"/>
+    <sheet name="Manny" sheetId="6" r:id="rId6"/>
+    <sheet name="Paul" sheetId="7" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="70">
   <si>
     <t>Use Case ID:</t>
   </si>
@@ -1521,7 +1525,7 @@
         <v>1</v>
       </c>
       <c r="D1" s="38">
-        <f>_xlfn.XLOOKUP($B$1,'Use case'!A:A,'Use case'!B:B,"",0,2)</f>
+        <f>_xlfn.XLOOKUP($B$1,'Use case template'!A:A,'Use case template'!B:B,"",0,2)</f>
         <v>0</v>
       </c>
     </row>
@@ -1530,14 +1534,14 @@
         <v>3</v>
       </c>
       <c r="B2" s="38">
-        <f>_xlfn.XLOOKUP($B$1,'Use case'!A:A,'Use case'!D:D,"",0,2)</f>
+        <f>_xlfn.XLOOKUP($B$1,'Use case template'!A:A,'Use case template'!D:D,"",0,2)</f>
         <v>0</v>
       </c>
       <c r="C2" s="33" t="s">
         <v>9</v>
       </c>
       <c r="D2" s="38">
-        <f>_xlfn.XLOOKUP($B$1,'Use case'!A:A,'Use case'!J:J,"",0,2)</f>
+        <f>_xlfn.XLOOKUP($B$1,'Use case template'!A:A,'Use case template'!J:J,"",0,2)</f>
         <v>0</v>
       </c>
       <c r="E2" s="1"/>
@@ -1547,7 +1551,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="39" t="str">
-        <f>IF(_xlfn.XLOOKUP($B$1,'Use case'!A:A,'Use case'!C:C,"",0,2)=0,"",_xlfn.XLOOKUP($B$1,'Use case'!A:A,'Use case'!C:C,"",0,2))</f>
+        <f>IF(_xlfn.XLOOKUP($B$1,'Use case template'!A:A,'Use case template'!C:C,"",0,2)=0,"",_xlfn.XLOOKUP($B$1,'Use case template'!A:A,'Use case template'!C:C,"",0,2))</f>
         <v/>
       </c>
       <c r="C3" s="39"/>
@@ -1558,7 +1562,7 @@
         <v>4</v>
       </c>
       <c r="B4" s="40">
-        <f>_xlfn.XLOOKUP($B$1,'Use case'!A:A,'Use case'!E:E,"",0,2)</f>
+        <f>_xlfn.XLOOKUP($B$1,'Use case template'!A:A,'Use case template'!E:E,"",0,2)</f>
         <v>0</v>
       </c>
       <c r="C4" s="40"/>
@@ -1571,7 +1575,7 @@
         <v>5</v>
       </c>
       <c r="B5" s="40">
-        <f>_xlfn.XLOOKUP($B$1,'Use case'!A:A,'Use case'!F:F,"",0,2)</f>
+        <f>_xlfn.XLOOKUP($B$1,'Use case template'!A:A,'Use case template'!F:F,"",0,2)</f>
         <v>0</v>
       </c>
       <c r="C5" s="40"/>
@@ -1584,7 +1588,7 @@
         <v>6</v>
       </c>
       <c r="B6" s="40">
-        <f>_xlfn.XLOOKUP($B$1,'Use case'!A:A,'Use case'!G:G,"",0,2)</f>
+        <f>_xlfn.XLOOKUP($B$1,'Use case template'!A:A,'Use case template'!G:G,"",0,2)</f>
         <v>0</v>
       </c>
       <c r="C6" s="40"/>
@@ -1597,7 +1601,7 @@
         <v>7</v>
       </c>
       <c r="B7" s="39">
-        <f>_xlfn.XLOOKUP($B$1,'Use case'!A:A,'Use case'!H:H,"",0,2)</f>
+        <f>_xlfn.XLOOKUP($B$1,'Use case template'!A:A,'Use case template'!H:H,"",0,2)</f>
         <v>0</v>
       </c>
       <c r="C7" s="39"/>
@@ -1608,7 +1612,7 @@
         <v>8</v>
       </c>
       <c r="B8" s="39">
-        <f>_xlfn.XLOOKUP($B$1,'Use case'!A:A,'Use case'!I:I,"",0,2)</f>
+        <f>_xlfn.XLOOKUP($B$1,'Use case template'!A:A,'Use case template'!I:I,"",0,2)</f>
         <v>0</v>
       </c>
       <c r="C8" s="39"/>
@@ -2065,4 +2069,784 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF01303C-A9D5-4728-85A1-B3B1654606BC}">
+  <dimension ref="A1:J26"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="9" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14" style="4" customWidth="1"/>
+    <col min="3" max="3" width="13.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="29.42578125" style="4" customWidth="1"/>
+    <col min="6" max="6" width="26.5703125" style="4" customWidth="1"/>
+    <col min="7" max="7" width="43.7109375" style="3" customWidth="1"/>
+    <col min="8" max="8" width="17" style="4" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.7109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.28515625" style="2" customWidth="1"/>
+    <col min="11" max="16384" width="9.140625" style="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" s="1" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C2" s="1"/>
+      <c r="G2" s="4"/>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="G3" s="4"/>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G4" s="4"/>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="G5" s="4"/>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="G6" s="4"/>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G7" s="4"/>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G8" s="4"/>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="G9" s="4"/>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G10" s="4"/>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="G11" s="4"/>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G12" s="4"/>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G13" s="4"/>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="G14" s="4"/>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G15" s="4"/>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A22" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A23" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A24" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A25" s="1" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A26" s="1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BED62618-10D4-4AC3-ACE9-FE527039EC52}">
+  <dimension ref="A1:J26"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="9" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14" style="4" customWidth="1"/>
+    <col min="3" max="3" width="13.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="29.42578125" style="4" customWidth="1"/>
+    <col min="6" max="6" width="26.5703125" style="4" customWidth="1"/>
+    <col min="7" max="7" width="43.7109375" style="3" customWidth="1"/>
+    <col min="8" max="8" width="17" style="4" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.7109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.28515625" style="2" customWidth="1"/>
+    <col min="11" max="16384" width="9.140625" style="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" s="1" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C2" s="1"/>
+      <c r="G2" s="4"/>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="G3" s="4"/>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G4" s="4"/>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="G5" s="4"/>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="G6" s="4"/>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G7" s="4"/>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G8" s="4"/>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="G9" s="4"/>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G10" s="4"/>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="G11" s="4"/>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G12" s="4"/>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G13" s="4"/>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="G14" s="4"/>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G15" s="4"/>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A22" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A23" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A24" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A25" s="1" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A26" s="1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1BFA99AA-42E4-4AD6-AE1A-F8BC73F53ED2}">
+  <dimension ref="A1:J26"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="9" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14" style="4" customWidth="1"/>
+    <col min="3" max="3" width="13.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="29.42578125" style="4" customWidth="1"/>
+    <col min="6" max="6" width="26.5703125" style="4" customWidth="1"/>
+    <col min="7" max="7" width="43.7109375" style="3" customWidth="1"/>
+    <col min="8" max="8" width="17" style="4" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.7109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.28515625" style="2" customWidth="1"/>
+    <col min="11" max="16384" width="9.140625" style="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" s="1" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C2" s="1"/>
+      <c r="G2" s="4"/>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="G3" s="4"/>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G4" s="4"/>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="G5" s="4"/>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="G6" s="4"/>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G7" s="4"/>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G8" s="4"/>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="G9" s="4"/>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G10" s="4"/>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="G11" s="4"/>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G12" s="4"/>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G13" s="4"/>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="G14" s="4"/>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G15" s="4"/>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A22" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A23" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A24" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A25" s="1" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A26" s="1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E19FFA8-B913-4564-BF18-E7CEF911FE02}">
+  <dimension ref="A1:J26"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="9" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14" style="4" customWidth="1"/>
+    <col min="3" max="3" width="13.85546875" style="3" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="29.42578125" style="4" customWidth="1"/>
+    <col min="6" max="6" width="26.5703125" style="4" customWidth="1"/>
+    <col min="7" max="7" width="43.7109375" style="3" customWidth="1"/>
+    <col min="8" max="8" width="17" style="4" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.7109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.28515625" style="2" customWidth="1"/>
+    <col min="11" max="16384" width="9.140625" style="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" s="1" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C2" s="1"/>
+      <c r="G2" s="4"/>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="G3" s="4"/>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G4" s="4"/>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="G5" s="4"/>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="G6" s="4"/>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G7" s="4"/>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G8" s="4"/>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="G9" s="4"/>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G10" s="4"/>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="G11" s="4"/>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G12" s="4"/>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G13" s="4"/>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="G14" s="4"/>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G15" s="4"/>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A22" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A23" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A24" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A25" s="1" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A26" s="1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>